<commit_message>
Add deposit actuals workbook, sources, and related task inputs.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/task/inputs/1 Balance Sheet Forecast.xlsx
+++ b/task/inputs/1 Balance Sheet Forecast.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cjwork/holodeck-archive/task/backtesting_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cjwork/holodeck-archive/task/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BE754A-5BE5-6F46-B073-6100AF35A589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21080" yWindow="1040" windowWidth="14760" windowHeight="20980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4920" yWindow="1040" windowWidth="30920" windowHeight="20980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Balance" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="Forecast Drivers" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>